<commit_message>
Timetable Pro: dynamic config, classroom timetables, frontend + API, conflict resolution
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/DATA/INPUT/classroom_data.xlsx
+++ b/DATA/INPUT/classroom_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ARISE-T.T-main\ARISE-T.T-main\iiitdwd_timetable_v2\DATA\INPUT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{331AB217-A7A1-48DF-ACF0-34E9AB73D8DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE1C782B-4445-4890-8F51-18B04475E81F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -489,7 +489,7 @@
         <v>13</v>
       </c>
       <c r="C8" s="1">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -500,7 +500,7 @@
         <v>15</v>
       </c>
       <c r="C9" s="1">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -511,7 +511,7 @@
         <v>15</v>
       </c>
       <c r="C10" s="1">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -566,7 +566,7 @@
         <v>13</v>
       </c>
       <c r="C15" s="1">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -577,7 +577,7 @@
         <v>15</v>
       </c>
       <c r="C16" s="1">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -588,7 +588,7 @@
         <v>15</v>
       </c>
       <c r="C17" s="1">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -643,7 +643,7 @@
         <v>29</v>
       </c>
       <c r="C22" s="1">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -654,7 +654,7 @@
         <v>29</v>
       </c>
       <c r="C23" s="1">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Organize repository for handover and archive generated artifacts.
Move historical outputs/logs into artifacts archive, add tests/docs/runbooks and input readmes, and keep repository root cleaner for maintainable day-to-day development.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/DATA/INPUT/classroom_data.xlsx
+++ b/DATA/INPUT/classroom_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ARISE-T.T-main\ARISE-T.T-main\iiitdwd_timetable_v2\DATA\INPUT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE1C782B-4445-4890-8F51-18B04475E81F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19BDF868-5B0D-4A8B-9475-5CFEAC0DF6CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -423,7 +423,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="1">
-        <v>116</v>
+        <v>136</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>